<commit_message>
feat(catholic): add lay core calendar source
</commit_message>
<xml_diff>
--- a/data/seed/calendar-rules.xlsx
+++ b/data/seed/calendar-rules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\MyAIProject\OBworkspace\codex\calrepo\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4472EA3A-35FD-460E-8124-D36DD9BA4F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C37640F-A2C2-40F6-B3FB-FD6D461086F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="先看这里" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="透视表1" sheetId="4" r:id="rId4"/>
     <sheet name="日历源目录" sheetId="2" r:id="rId5"/>
     <sheet name="透视表2" sheetId="5" r:id="rId6"/>
-    <sheet name="节日总表" sheetId="3" r:id="rId7"/>
+    <sheet name="天主教罗马礼规则" sheetId="8" r:id="rId7"/>
+    <sheet name="节日总表" sheetId="3" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">二十四节气!$A$3:$J$27</definedName>
@@ -27,14 +28,14 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId8"/>
-    <pivotCache cacheId="1" r:id="rId9"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
+    <pivotCache cacheId="1" r:id="rId10"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6049" uniqueCount="1779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6202" uniqueCount="1839">
   <si>
     <t>CalRepo 日历规则数据库</t>
   </si>
@@ -5582,6 +5583,186 @@
   </si>
   <si>
     <t>公历 12-10</t>
+  </si>
+  <si>
+    <t>KeepOn 采用优先级</t>
+  </si>
+  <si>
+    <t>3（弃用）</t>
+  </si>
+  <si>
+    <t>2（外部候选）</t>
+  </si>
+  <si>
+    <t>1（CalRepo 已发布）</t>
+  </si>
+  <si>
+    <t>SRC-CATHOLIC-LAITY-CORE</t>
+  </si>
+  <si>
+    <t>天主教教友核心日历</t>
+  </si>
+  <si>
+    <t>普通天主教教友</t>
+  </si>
+  <si>
+    <t>天主教（罗马礼）</t>
+  </si>
+  <si>
+    <t>待发布</t>
+  </si>
+  <si>
+    <t>规则基于通用罗马礼；待生成和跨年核验。</t>
+  </si>
+  <si>
+    <t>核心大节与核心圣人规则待发布</t>
+  </si>
+  <si>
+    <t>生成 ICS 并核验</t>
+  </si>
+  <si>
+    <t>SRC-CATHOLIC-GENERAL-ROMAN</t>
+  </si>
+  <si>
+    <t>天主教通用罗马礼完整日历</t>
+  </si>
+  <si>
+    <t>神职、修会、礼仪研究及需要完整资料者</t>
+  </si>
+  <si>
+    <t>https://calrepo.com/ical/v1/religion/catholic-general-roman/en.ics</t>
+  </si>
+  <si>
+    <t>A：已公开版本化 ICS；完整版包含年度礼仪与通用圣人。</t>
+  </si>
+  <si>
+    <t>已发布；重点高亮由天主教罗马礼规则表决定。</t>
+  </si>
+  <si>
+    <t>年度复核上游与核心规则</t>
+  </si>
+  <si>
+    <t>规则值</t>
+  </si>
+  <si>
+    <t>教友核心</t>
+  </si>
+  <si>
+    <t>完整版高亮</t>
+  </si>
+  <si>
+    <t>中文说明</t>
+  </si>
+  <si>
+    <t>英文说明</t>
+  </si>
+  <si>
+    <t>依据</t>
+  </si>
+  <si>
+    <t>CATH-001</t>
+  </si>
+  <si>
+    <t>minimum_grade</t>
+  </si>
+  <si>
+    <t>隆重节日及主要礼仪节点</t>
+  </si>
+  <si>
+    <t>Solemnities and major liturgical observances</t>
+  </si>
+  <si>
+    <t>Liturgical Calendar API grade</t>
+  </si>
+  <si>
+    <t>核心版不纳入守夜弥撒</t>
+  </si>
+  <si>
+    <t>CATH-002</t>
+  </si>
+  <si>
+    <t>exclude_key_suffix</t>
+  </si>
+  <si>
+    <t>_vigil</t>
+  </si>
+  <si>
+    <t>排除守夜弥撒重复条目</t>
+  </si>
+  <si>
+    <t>Exclude vigil Mass duplicates</t>
+  </si>
+  <si>
+    <t>Editorial policy</t>
+  </si>
+  <si>
+    <t>CATH-003</t>
+  </si>
+  <si>
+    <t>event_key</t>
+  </si>
+  <si>
+    <t>StFrancisAssisi</t>
+  </si>
+  <si>
+    <t>亚西西的圣方济各</t>
+  </si>
+  <si>
+    <t>Saint Francis of Assisi</t>
+  </si>
+  <si>
+    <t>General Roman Calendar</t>
+  </si>
+  <si>
+    <t>核心圣人</t>
+  </si>
+  <si>
+    <t>CATH-004</t>
+  </si>
+  <si>
+    <t>StThereseChildJesus</t>
+  </si>
+  <si>
+    <t>圣女小德兰</t>
+  </si>
+  <si>
+    <t>Saint Therese of the Child Jesus</t>
+  </si>
+  <si>
+    <t>CATH-005</t>
+  </si>
+  <si>
+    <t>StAugustine</t>
+  </si>
+  <si>
+    <t>圣奥思定</t>
+  </si>
+  <si>
+    <t>Saint Augustine</t>
+  </si>
+  <si>
+    <t>CATH-006</t>
+  </si>
+  <si>
+    <t>StFrancisXavier</t>
+  </si>
+  <si>
+    <t>圣方济各沙勿略</t>
+  </si>
+  <si>
+    <t>Saint Francis Xavier</t>
+  </si>
+  <si>
+    <t>CATH-007</t>
+  </si>
+  <si>
+    <t>StMaryMagdalene</t>
+  </si>
+  <si>
+    <t>圣玛利亚玛达肋纳</t>
+  </si>
+  <si>
+    <t>Saint Mary Magdalene</t>
   </si>
 </sst>
 </file>
@@ -5860,11 +6041,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -12555,15 +12736,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CalendarSourceRegistry" displayName="CalendarSourceRegistry" ref="A1:U42" totalsRowShown="0">
-  <autoFilter ref="A1:U42" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="CalendarSourceRegistry" displayName="CalendarSourceRegistry" ref="A1:V42" totalsRowShown="0">
+  <autoFilter ref="A1:V42" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="4">
       <filters>
         <filter val="中国"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="21">
+  <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="源编号"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="一级分类"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="日历源名称"/>
@@ -12585,6 +12766,7 @@
     <tableColumn id="19" xr3:uid="{0A12A09D-0014-4DBF-BE95-EA9DFA7B0F85}" name="生命周期"/>
     <tableColumn id="20" xr3:uid="{E077B5D5-EBDF-4C35-88FA-430EEC6820CF}" name="发布状态"/>
     <tableColumn id="21" xr3:uid="{00E251B1-9870-470C-8002-C9F5E8B9EE70}" name="弃用原因"/>
+    <tableColumn id="22" xr3:uid="{7033D850-7397-43CA-A725-BF90DD5922A8}" name="KeepOn 采用优先级"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12820,10 +13002,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="27.95" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
+      <c r="B1" s="31"/>
     </row>
     <row r="3" spans="1:2" ht="28.5">
       <c r="A3" s="1" t="s">
@@ -12949,30 +13131,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>1493</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>1494</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
     </row>
     <row r="3" spans="1:10" s="27" customFormat="1" ht="15">
       <c r="A3" s="27" t="s">
@@ -13564,32 +13746,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>1455</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>1456</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:11" s="27" customFormat="1" ht="15">
       <c r="A3" s="27" t="s">
@@ -15200,7 +15382,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U45"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -15221,9 +15403,10 @@
     <col min="19" max="19" width="9.625" customWidth="1"/>
     <col min="20" max="20" width="8.375" customWidth="1"/>
     <col min="21" max="21" width="12.25" customWidth="1"/>
+    <col min="22" max="22" width="22.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15">
+    <row r="1" spans="1:22" ht="15">
       <c r="A1" s="13" t="s">
         <v>23</v>
       </c>
@@ -15287,8 +15470,11 @@
       <c r="U1" t="s">
         <v>1650</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="57">
+      <c r="V1" t="s">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="57">
       <c r="A2" s="16" t="s">
         <v>40</v>
       </c>
@@ -15348,8 +15534,11 @@
       <c r="U2" t="s">
         <v>1654</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" ht="28.5" hidden="1">
+      <c r="V2" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="28.5" hidden="1">
       <c r="A3" s="16" t="s">
         <v>52</v>
       </c>
@@ -15397,8 +15586,11 @@
       <c r="Q3" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" ht="28.5" hidden="1">
+      <c r="V3" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="28.5" hidden="1">
       <c r="A4" s="16" t="s">
         <v>59</v>
       </c>
@@ -15446,8 +15638,11 @@
       <c r="Q4" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" ht="28.5" hidden="1">
+      <c r="V4" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="28.5" hidden="1">
       <c r="A5" s="16" t="s">
         <v>64</v>
       </c>
@@ -15495,8 +15690,11 @@
       <c r="Q5" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" ht="28.5" hidden="1">
+      <c r="V5" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="28.5" hidden="1">
       <c r="A6" s="16" t="s">
         <v>69</v>
       </c>
@@ -15544,8 +15742,11 @@
       <c r="Q6" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" ht="28.5" hidden="1">
+      <c r="V6" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="28.5" hidden="1">
       <c r="A7" s="16" t="s">
         <v>74</v>
       </c>
@@ -15593,8 +15794,11 @@
       <c r="Q7" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" ht="28.5" hidden="1">
+      <c r="V7" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="28.5" hidden="1">
       <c r="A8" s="16" t="s">
         <v>79</v>
       </c>
@@ -15642,8 +15846,11 @@
       <c r="Q8" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" ht="28.5" hidden="1">
+      <c r="V8" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="28.5" hidden="1">
       <c r="A9" s="16" t="s">
         <v>84</v>
       </c>
@@ -15691,8 +15898,11 @@
       <c r="Q9" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" ht="28.5" hidden="1">
+      <c r="V9" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="28.5" hidden="1">
       <c r="A10" s="16" t="s">
         <v>89</v>
       </c>
@@ -15740,8 +15950,11 @@
       <c r="Q10" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" ht="28.5" hidden="1">
+      <c r="V10" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="28.5" hidden="1">
       <c r="A11" s="16" t="s">
         <v>94</v>
       </c>
@@ -15789,8 +16002,11 @@
       <c r="Q11" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" ht="28.5" hidden="1">
+      <c r="V11" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="28.5" hidden="1">
       <c r="A12" s="16" t="s">
         <v>99</v>
       </c>
@@ -15838,8 +16054,11 @@
       <c r="Q12" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" ht="28.5" hidden="1">
+      <c r="V12" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="28.5" hidden="1">
       <c r="A13" s="16" t="s">
         <v>105</v>
       </c>
@@ -15887,8 +16106,11 @@
       <c r="Q13" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" ht="28.5" hidden="1">
+      <c r="V13" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="28.5" hidden="1">
       <c r="A14" s="16" t="s">
         <v>111</v>
       </c>
@@ -15936,8 +16158,11 @@
       <c r="Q14" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" ht="28.5" hidden="1">
+      <c r="V14" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="28.5" hidden="1">
       <c r="A15" s="16" t="s">
         <v>118</v>
       </c>
@@ -15985,8 +16210,11 @@
       <c r="Q15" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" ht="28.5" hidden="1">
+      <c r="V15" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" ht="28.5" hidden="1">
       <c r="A16" s="16" t="s">
         <v>124</v>
       </c>
@@ -16034,8 +16262,11 @@
       <c r="Q16" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" ht="28.5" hidden="1">
+      <c r="V16" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" ht="28.5" hidden="1">
       <c r="A17" s="16" t="s">
         <v>129</v>
       </c>
@@ -16083,8 +16314,11 @@
       <c r="Q17" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" ht="28.5" hidden="1">
+      <c r="V17" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="28.5" hidden="1">
       <c r="A18" s="16" t="s">
         <v>134</v>
       </c>
@@ -16134,8 +16368,11 @@
       <c r="Q18" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" ht="57">
+      <c r="V18" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" ht="57">
       <c r="A19" s="16" t="s">
         <v>141</v>
       </c>
@@ -16197,8 +16434,11 @@
       <c r="U19" t="s">
         <v>1654</v>
       </c>
-    </row>
-    <row r="20" spans="1:21" ht="57">
+      <c r="V19" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="57">
       <c r="A20" s="16" t="s">
         <v>153</v>
       </c>
@@ -16260,8 +16500,11 @@
       <c r="U20" t="s">
         <v>1654</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" ht="57">
+      <c r="V20" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="57">
       <c r="A21" s="16" t="s">
         <v>159</v>
       </c>
@@ -16321,8 +16564,11 @@
       <c r="U21" t="s">
         <v>1654</v>
       </c>
-    </row>
-    <row r="22" spans="1:21" ht="28.5" hidden="1">
+      <c r="V21" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" ht="28.5" hidden="1">
       <c r="A22" s="16" t="s">
         <v>167</v>
       </c>
@@ -16370,8 +16616,11 @@
       <c r="Q22" s="17" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23" spans="1:21" ht="42.75" hidden="1">
+      <c r="V22" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" ht="42.75" hidden="1">
       <c r="A23" s="16" t="s">
         <v>1372</v>
       </c>
@@ -16421,8 +16670,11 @@
       <c r="Q23" s="25">
         <v>46227</v>
       </c>
-    </row>
-    <row r="24" spans="1:21" ht="28.5" hidden="1">
+      <c r="V23" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" ht="28.5" hidden="1">
       <c r="A24" s="16" t="s">
         <v>181</v>
       </c>
@@ -16470,8 +16722,11 @@
       <c r="Q24" s="17" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="25" spans="1:21" ht="57" hidden="1">
+      <c r="V24" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" ht="57" hidden="1">
       <c r="A25" s="16" t="s">
         <v>191</v>
       </c>
@@ -16530,8 +16785,11 @@
       <c r="T25" t="s">
         <v>1722</v>
       </c>
-    </row>
-    <row r="26" spans="1:21" ht="28.5" hidden="1">
+      <c r="V25" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" ht="28.5" hidden="1">
       <c r="A26" s="16" t="s">
         <v>192</v>
       </c>
@@ -16581,8 +16839,11 @@
       <c r="Q26" s="17" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="27" spans="1:21" ht="28.5" hidden="1">
+      <c r="V26" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" ht="28.5" hidden="1">
       <c r="A27" s="16" t="s">
         <v>202</v>
       </c>
@@ -16632,8 +16893,11 @@
       <c r="Q27" s="17" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="28" spans="1:21" ht="28.5" hidden="1">
+      <c r="V27" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" ht="28.5" hidden="1">
       <c r="A28" s="16" t="s">
         <v>212</v>
       </c>
@@ -16683,8 +16947,11 @@
       <c r="Q28" s="17" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="29" spans="1:21" ht="42.75" hidden="1">
+      <c r="V28" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" ht="42.75" hidden="1">
       <c r="A29" s="16" t="s">
         <v>221</v>
       </c>
@@ -16743,8 +17010,11 @@
       <c r="T29" t="s">
         <v>1722</v>
       </c>
-    </row>
-    <row r="30" spans="1:21" ht="42.75" hidden="1">
+      <c r="V29" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" ht="42.75" hidden="1">
       <c r="A30" s="16" t="s">
         <v>228</v>
       </c>
@@ -16803,8 +17073,11 @@
       <c r="T30" t="s">
         <v>1722</v>
       </c>
-    </row>
-    <row r="31" spans="1:21">
+      <c r="V30" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31" s="16" t="s">
         <v>233</v>
       </c>
@@ -16852,8 +17125,11 @@
       <c r="Q31" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="32" spans="1:21">
+      <c r="V31" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" s="16" t="s">
         <v>243</v>
       </c>
@@ -16903,8 +17179,11 @@
       <c r="Q32" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="33" spans="1:20">
+      <c r="V32" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22">
       <c r="A33" s="16" t="s">
         <v>250</v>
       </c>
@@ -16954,8 +17233,11 @@
       <c r="Q33" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="34" spans="1:20">
+      <c r="V33" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22">
       <c r="A34" s="16" t="s">
         <v>255</v>
       </c>
@@ -17003,8 +17285,11 @@
       <c r="Q34" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="35" spans="1:20">
+      <c r="V34" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22">
       <c r="A35" s="16" t="s">
         <v>263</v>
       </c>
@@ -17052,8 +17337,11 @@
       <c r="Q35" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="36" spans="1:20">
+      <c r="V35" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22">
       <c r="A36" s="16" t="s">
         <v>270</v>
       </c>
@@ -17101,8 +17389,11 @@
       <c r="Q36" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="37" spans="1:20">
+      <c r="V36" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22">
       <c r="A37" s="16" t="s">
         <v>278</v>
       </c>
@@ -17150,8 +17441,11 @@
       <c r="Q37" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="38" spans="1:20">
+      <c r="V37" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38" s="16" t="s">
         <v>283</v>
       </c>
@@ -17201,8 +17495,11 @@
       <c r="Q38" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="39" spans="1:20">
+      <c r="V38" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22">
       <c r="A39" s="16" t="s">
         <v>292</v>
       </c>
@@ -17250,8 +17547,11 @@
       <c r="Q39" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="40" spans="1:20">
+      <c r="V39" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40" s="18" t="s">
         <v>300</v>
       </c>
@@ -17299,8 +17599,11 @@
       <c r="Q40" s="20" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="41" spans="1:20" ht="42.75" hidden="1">
+      <c r="V40" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" ht="42.75" hidden="1">
       <c r="A41" s="12" t="s">
         <v>1387</v>
       </c>
@@ -17350,8 +17653,11 @@
       <c r="Q41" s="26">
         <v>46227</v>
       </c>
-    </row>
-    <row r="42" spans="1:20" ht="57" hidden="1">
+      <c r="V41" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" ht="57" hidden="1">
       <c r="A42" s="12" t="s">
         <v>1394</v>
       </c>
@@ -17401,8 +17707,11 @@
       <c r="Q42" s="26">
         <v>46227</v>
       </c>
-    </row>
-    <row r="43" spans="1:20" ht="42.75">
+      <c r="V42" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" ht="42.75">
       <c r="A43" s="16" t="s">
         <v>1661</v>
       </c>
@@ -17461,8 +17770,11 @@
       <c r="T43" t="s">
         <v>1733</v>
       </c>
-    </row>
-    <row r="44" spans="1:20" ht="28.5">
+      <c r="V43" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" ht="28.5">
       <c r="A44" s="16" t="s">
         <v>1668</v>
       </c>
@@ -17521,8 +17833,11 @@
       <c r="T44" t="s">
         <v>1733</v>
       </c>
-    </row>
-    <row r="45" spans="1:20">
+      <c r="V44" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22">
       <c r="A45" t="s">
         <v>1735</v>
       </c>
@@ -17565,7 +17880,7 @@
       <c r="P45" t="s">
         <v>1741</v>
       </c>
-      <c r="Q45" s="32">
+      <c r="Q45" s="30">
         <v>46228</v>
       </c>
       <c r="R45" t="s">
@@ -17576,6 +17891,130 @@
       </c>
       <c r="T45" t="s">
         <v>1722</v>
+      </c>
+      <c r="V45" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22">
+      <c r="A46" t="s">
+        <v>1783</v>
+      </c>
+      <c r="B46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1784</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E46" t="s">
+        <v>137</v>
+      </c>
+      <c r="F46" t="s">
+        <v>1786</v>
+      </c>
+      <c r="H46" t="s">
+        <v>56</v>
+      </c>
+      <c r="I46" t="s">
+        <v>1787</v>
+      </c>
+      <c r="K46" t="s">
+        <v>1717</v>
+      </c>
+      <c r="L46" t="s">
+        <v>1788</v>
+      </c>
+      <c r="M46" t="s">
+        <v>44</v>
+      </c>
+      <c r="N46" t="s">
+        <v>177</v>
+      </c>
+      <c r="O46" t="s">
+        <v>1789</v>
+      </c>
+      <c r="P46" t="s">
+        <v>1790</v>
+      </c>
+      <c r="Q46" s="30">
+        <v>46229</v>
+      </c>
+      <c r="R46" t="s">
+        <v>1666</v>
+      </c>
+      <c r="S46" t="s">
+        <v>1667</v>
+      </c>
+      <c r="T46" t="s">
+        <v>1787</v>
+      </c>
+      <c r="V46" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22">
+      <c r="A47" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B47" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1792</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1793</v>
+      </c>
+      <c r="E47" t="s">
+        <v>137</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1786</v>
+      </c>
+      <c r="H47" t="s">
+        <v>56</v>
+      </c>
+      <c r="I47" t="s">
+        <v>44</v>
+      </c>
+      <c r="J47" t="s">
+        <v>1794</v>
+      </c>
+      <c r="K47" t="s">
+        <v>1717</v>
+      </c>
+      <c r="L47" t="s">
+        <v>1795</v>
+      </c>
+      <c r="M47" t="s">
+        <v>44</v>
+      </c>
+      <c r="N47" t="s">
+        <v>177</v>
+      </c>
+      <c r="O47" t="s">
+        <v>1796</v>
+      </c>
+      <c r="P47" t="s">
+        <v>1797</v>
+      </c>
+      <c r="Q47" s="30">
+        <v>46229</v>
+      </c>
+      <c r="R47" t="s">
+        <v>1666</v>
+      </c>
+      <c r="S47" t="s">
+        <v>1667</v>
+      </c>
+      <c r="T47" t="s">
+        <v>1722</v>
+      </c>
+      <c r="V47" t="s">
+        <v>1782</v>
       </c>
     </row>
   </sheetData>
@@ -17801,6 +18240,281 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4ECD824-7211-4591-B934-1B096D87B557}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="27" customFormat="1" ht="15">
+      <c r="A1" s="27" t="s">
+        <v>1457</v>
+      </c>
+      <c r="B1" s="27" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>1798</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>1799</v>
+      </c>
+      <c r="E1" s="27" t="s">
+        <v>1800</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>1801</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>1802</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>1803</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>315</v>
+      </c>
+      <c r="J1" s="27" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1805</v>
+      </c>
+      <c r="C2">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1806</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1807</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1808</v>
+      </c>
+      <c r="I2" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1809</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>1810</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1811</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1812</v>
+      </c>
+      <c r="D3" t="s">
+        <v>172</v>
+      </c>
+      <c r="E3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1813</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1814</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1815</v>
+      </c>
+      <c r="I3" s="30">
+        <v>46229</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>1816</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1818</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1819</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1820</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="I4" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J4" t="s">
+        <v>1822</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1824</v>
+      </c>
+      <c r="D5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1825</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1826</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1821</v>
+      </c>
+      <c r="I5" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1822</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>1827</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1828</v>
+      </c>
+      <c r="D6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1829</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1830</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1821</v>
+      </c>
+      <c r="I6" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1822</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1832</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1833</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1834</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1821</v>
+      </c>
+      <c r="I7" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J7" t="s">
+        <v>1822</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>1835</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1836</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1837</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1838</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1821</v>
+      </c>
+      <c r="I8" s="30">
+        <v>46229</v>
+      </c>
+      <c r="J8" t="s">
+        <v>1822</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:R362"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -33023,7 +33737,7 @@
       <c r="K346" t="s">
         <v>549</v>
       </c>
-      <c r="L346" s="32">
+      <c r="L346" s="30">
         <v>46228</v>
       </c>
       <c r="M346" t="s">
@@ -33076,7 +33790,7 @@
       <c r="K347" t="s">
         <v>549</v>
       </c>
-      <c r="L347" s="32">
+      <c r="L347" s="30">
         <v>46228</v>
       </c>
       <c r="M347" t="s">
@@ -33129,7 +33843,7 @@
       <c r="K348" t="s">
         <v>549</v>
       </c>
-      <c r="L348" s="32">
+      <c r="L348" s="30">
         <v>46228</v>
       </c>
       <c r="M348" t="s">
@@ -33182,7 +33896,7 @@
       <c r="K349" t="s">
         <v>549</v>
       </c>
-      <c r="L349" s="32">
+      <c r="L349" s="30">
         <v>46228</v>
       </c>
       <c r="M349" t="s">
@@ -33235,7 +33949,7 @@
       <c r="K350" t="s">
         <v>549</v>
       </c>
-      <c r="L350" s="32">
+      <c r="L350" s="30">
         <v>46228</v>
       </c>
       <c r="M350" t="s">
@@ -33288,7 +34002,7 @@
       <c r="K351" t="s">
         <v>549</v>
       </c>
-      <c r="L351" s="32">
+      <c r="L351" s="30">
         <v>46228</v>
       </c>
       <c r="M351" t="s">
@@ -33341,7 +34055,7 @@
       <c r="K352" t="s">
         <v>549</v>
       </c>
-      <c r="L352" s="32">
+      <c r="L352" s="30">
         <v>46228</v>
       </c>
       <c r="M352" t="s">
@@ -33394,7 +34108,7 @@
       <c r="K353" t="s">
         <v>549</v>
       </c>
-      <c r="L353" s="32">
+      <c r="L353" s="30">
         <v>46228</v>
       </c>
       <c r="M353" t="s">
@@ -33447,7 +34161,7 @@
       <c r="K354" t="s">
         <v>549</v>
       </c>
-      <c r="L354" s="32">
+      <c r="L354" s="30">
         <v>46228</v>
       </c>
       <c r="M354" t="s">
@@ -33500,7 +34214,7 @@
       <c r="K355" t="s">
         <v>549</v>
       </c>
-      <c r="L355" s="32">
+      <c r="L355" s="30">
         <v>46228</v>
       </c>
       <c r="M355" t="s">
@@ -33553,7 +34267,7 @@
       <c r="K356" t="s">
         <v>549</v>
       </c>
-      <c r="L356" s="32">
+      <c r="L356" s="30">
         <v>46228</v>
       </c>
       <c r="M356" t="s">
@@ -33606,7 +34320,7 @@
       <c r="K357" t="s">
         <v>549</v>
       </c>
-      <c r="L357" s="32">
+      <c r="L357" s="30">
         <v>46228</v>
       </c>
       <c r="M357" t="s">
@@ -33659,7 +34373,7 @@
       <c r="K358" t="s">
         <v>549</v>
       </c>
-      <c r="L358" s="32">
+      <c r="L358" s="30">
         <v>46228</v>
       </c>
       <c r="M358" t="s">
@@ -33712,7 +34426,7 @@
       <c r="K359" t="s">
         <v>549</v>
       </c>
-      <c r="L359" s="32">
+      <c r="L359" s="30">
         <v>46228</v>
       </c>
       <c r="M359" t="s">
@@ -33765,7 +34479,7 @@
       <c r="K360" t="s">
         <v>549</v>
       </c>
-      <c r="L360" s="32">
+      <c r="L360" s="30">
         <v>46228</v>
       </c>
       <c r="M360" t="s">
@@ -33818,7 +34532,7 @@
       <c r="K361" t="s">
         <v>549</v>
       </c>
-      <c r="L361" s="32">
+      <c r="L361" s="30">
         <v>46228</v>
       </c>
       <c r="M361" t="s">
@@ -33871,7 +34585,7 @@
       <c r="K362" t="s">
         <v>549</v>
       </c>
-      <c r="L362" s="32">
+      <c r="L362" s="30">
         <v>46228</v>
       </c>
       <c r="M362" t="s">

</xml_diff>